<commit_message>
auto(MT): 3h refresh 2026-05-20T10:05Z
</commit_message>
<xml_diff>
--- a/daily_report_mt_2026-05-20.xlsx
+++ b/daily_report_mt_2026-05-20.xlsx
@@ -727,7 +727,6 @@
           <t>PL</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
           <t>David Caruana</t>
@@ -753,8 +752,6 @@
           <t>2026-05-18</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
       <c r="M3" t="inlineStr">
         <is>
           <t>2026-05-17</t>
@@ -989,7 +986,6 @@
           <t>PL</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
           <t>David Caruana</t>
@@ -1099,7 +1095,6 @@
           <t>PL</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
           <t>David Caruana</t>
@@ -1209,7 +1204,6 @@
           <t>PL</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
           <t>Anthony Agius Decelis</t>
@@ -1235,8 +1229,6 @@
           <t>2026-05-17</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
       <c r="M7" t="inlineStr">
         <is>
           <t>2026-05-20 08:55</t>
@@ -1301,7 +1293,6 @@
           <t>PL</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr">
         <is>
           <t>Anthony Agius Decelis</t>
@@ -1327,8 +1318,6 @@
           <t>2026-05-17</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
       <c r="M9" t="inlineStr">
         <is>
           <t>2026-05-20 08:55</t>

</xml_diff>

<commit_message>
auto(MT): 3h refresh 2026-05-20T16:23Z
</commit_message>
<xml_diff>
--- a/daily_report_mt_2026-05-20.xlsx
+++ b/daily_report_mt_2026-05-20.xlsx
@@ -559,14 +559,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N4"/>
+  <dimension ref="A1:N5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
     <col width="7" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
-    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
     <col width="9" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
@@ -827,11 +827,60 @@
         <v>2</v>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Julian Borg</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>PN</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Julian Borg</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>1545088225724311</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>1337673231567873</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="N5" t="n">
+        <v>9</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G3" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G5" r:id="rId4"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -843,7 +892,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M10"/>
+  <dimension ref="A1:M11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
@@ -1375,6 +1424,51 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Julian Borg</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>PN</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr"/>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Julian Borg</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>1545088225724311</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>1337673231567873</t>
+        </is>
+      </c>
+      <c r="G11" s="5" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>2026-05-20 16:20</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G2" r:id="rId1"/>
@@ -1386,6 +1480,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G8" r:id="rId7"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G9" r:id="rId8"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G11" r:id="rId10"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>